<commit_message>
re-badge the home market to india and read values as inr
no rate conversion, so every figure keeps its original magnitude; the
readiness sheet states the source dataset so the provenance is on record
</commit_message>
<xml_diff>
--- a/excel/data_audit.xlsx
+++ b/excel/data_audit.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="243">
   <si>
     <t>Online Retail II: data readiness sign-off</t>
   </si>
@@ -60,6 +60,9 @@
     <t>My readiness verdict</t>
   </si>
   <si>
+    <t>I built this on the UCI Online Retail II transactional dataset, re-badged to an Indian retail context with values read as INR and no rate conversion applied. The transaction grain, product catalogue and customer behaviour are the source data's.</t>
+  </si>
+  <si>
     <t>The data is usable once I deal with a few known problems: 243,007 rows have no customer, 34,337 rows are exact duplicates and 6,207 rows carry a price of zero or less.</t>
   </si>
   <si>
@@ -294,10 +297,10 @@
     <t>Customers</t>
   </si>
   <si>
-    <t>United Kingdom</t>
-  </si>
-  <si>
-    <t>EIRE</t>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Ireland</t>
   </si>
   <si>
     <t>Netherlands</t>
@@ -387,7 +390,7 @@
     <t>Canada</t>
   </si>
   <si>
-    <t>RSA</t>
+    <t>South Africa</t>
   </si>
   <si>
     <t>Thailand</t>
@@ -408,7 +411,7 @@
     <t>Bermuda</t>
   </si>
   <si>
-    <t>Korea</t>
+    <t>South Korea</t>
   </si>
   <si>
     <t>Czech Republic</t>
@@ -753,7 +756,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;₹&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.00%"/>
   </numFmts>
   <fonts count="4">
@@ -847,7 +850,7 @@
       <numFmt numFmtId="166" formatCode="0.00%"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#,##0.00"/>
+      <numFmt numFmtId="165" formatCode="&quot;₹&quot;#,##0.00"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1180,10 +1183,10 @@
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>United Kingdom</c:v>
+                  <c:v>India</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>EIRE</c:v>
+                  <c:v>Ireland</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Netherlands</c:v>
@@ -1796,7 +1799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="52.7109375" customWidth="1"/>
@@ -1909,13 +1912,21 @@
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
     </row>
+    <row r="16" spans="1:3" ht="32" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1942,39 +1953,39 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2" s="8">
         <v>1067371</v>
@@ -1994,10 +2005,10 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
         <v>29</v>
-      </c>
-      <c r="B3" t="s">
-        <v>28</v>
       </c>
       <c r="C3" s="8">
         <v>1067371</v>
@@ -2017,10 +2028,10 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="8">
         <v>1062989</v>
@@ -2040,10 +2051,10 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="8">
         <v>1067371</v>
@@ -2069,10 +2080,10 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" s="8">
         <v>1067371</v>
@@ -2092,10 +2103,10 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" s="8">
         <v>1067371</v>
@@ -2121,10 +2132,10 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
         <v>38</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
       </c>
       <c r="C8" s="8">
         <v>824364</v>
@@ -2150,10 +2161,10 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" s="8">
         <v>1067371</v>
@@ -2173,10 +2184,10 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" s="8">
         <v>1067371</v>
@@ -2215,21 +2226,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B2" s="8">
         <v>243007</v>
@@ -2238,12 +2249,12 @@
         <v>0.2276687299917273</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" s="8">
         <v>4382</v>
@@ -2252,12 +2263,12 @@
         <v>0.004105414143723222</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B4" s="8">
         <v>19494</v>
@@ -2266,12 +2277,12 @@
         <v>0.01826356533951175</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B5" s="8">
         <v>34337</v>
@@ -2280,12 +2291,12 @@
         <v>0.03216969544797451</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B6" s="8">
         <v>6207</v>
@@ -2294,12 +2305,12 @@
         <v>0.005815222635803296</v>
       </c>
       <c r="D6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B7" s="8">
         <v>0</v>
@@ -2308,12 +2319,12 @@
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" s="8">
         <v>3457</v>
@@ -2322,12 +2333,12 @@
         <v>0.003238798880614144</v>
       </c>
       <c r="D8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B9" s="8">
         <v>5811</v>
@@ -2336,12 +2347,12 @@
         <v>0.005444217615056058</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B10" s="8">
         <v>3472</v>
@@ -2350,7 +2361,7 @@
         <v>0.003252852101096995</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2372,18 +2383,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2" s="8">
         <v>45228</v>
@@ -2394,7 +2405,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B3" s="8">
         <v>31555</v>
@@ -2405,7 +2416,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B4" s="8">
         <v>29388</v>
@@ -2416,7 +2427,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B5" s="8">
         <v>41511</v>
@@ -2427,7 +2438,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B6" s="8">
         <v>34057</v>
@@ -2438,7 +2449,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B7" s="8">
         <v>35323</v>
@@ -2449,7 +2460,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8" s="8">
         <v>39983</v>
@@ -2460,7 +2471,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B9" s="8">
         <v>33383</v>
@@ -2471,7 +2482,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B10" s="8">
         <v>33306</v>
@@ -2482,7 +2493,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B11" s="8">
         <v>42091</v>
@@ -2493,7 +2504,7 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B12" s="8">
         <v>59098</v>
@@ -2504,7 +2515,7 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B13" s="8">
         <v>78015</v>
@@ -2515,7 +2526,7 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B14" s="8">
         <v>65004</v>
@@ -2526,7 +2537,7 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B15" s="8">
         <v>35147</v>
@@ -2537,7 +2548,7 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B16" s="8">
         <v>27707</v>
@@ -2548,7 +2559,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B17" s="8">
         <v>36748</v>
@@ -2559,7 +2570,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B18" s="8">
         <v>29916</v>
@@ -2570,7 +2581,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B19" s="8">
         <v>37030</v>
@@ -2581,7 +2592,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B20" s="8">
         <v>36874</v>
@@ -2592,7 +2603,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B21" s="8">
         <v>39518</v>
@@ -2603,7 +2614,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B22" s="8">
         <v>35284</v>
@@ -2614,7 +2625,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B23" s="8">
         <v>50226</v>
@@ -2625,7 +2636,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B24" s="8">
         <v>60742</v>
@@ -2636,7 +2647,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B25" s="8">
         <v>84711</v>
@@ -2647,7 +2658,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B26" s="8">
         <v>25526</v>
@@ -2678,21 +2689,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B2" s="8">
         <v>981330</v>
@@ -2706,7 +2717,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B3" s="8">
         <v>17866</v>
@@ -2720,7 +2731,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B4" s="8">
         <v>5140</v>
@@ -2734,7 +2745,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B5" s="8">
         <v>17624</v>
@@ -2748,7 +2759,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B6" s="8">
         <v>14330</v>
@@ -2762,7 +2773,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B7" s="8">
         <v>1913</v>
@@ -2776,7 +2787,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B8" s="8">
         <v>3189</v>
@@ -2790,7 +2801,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B9" s="8">
         <v>3811</v>
@@ -2804,7 +2815,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B10" s="8">
         <v>1364</v>
@@ -2818,7 +2829,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B11" s="8">
         <v>817</v>
@@ -2832,7 +2843,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B12" s="8">
         <v>3123</v>
@@ -2846,7 +2857,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B13" s="8">
         <v>2620</v>
@@ -2860,7 +2871,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B14" s="8">
         <v>582</v>
@@ -2874,7 +2885,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B15" s="8">
         <v>1664</v>
@@ -2888,7 +2899,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B16" s="8">
         <v>1455</v>
@@ -2902,7 +2913,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B17" s="8">
         <v>1534</v>
@@ -2916,7 +2927,7 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B18" s="8">
         <v>1049</v>
@@ -2930,7 +2941,7 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B19" s="8">
         <v>1176</v>
@@ -2944,7 +2955,7 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B20" s="8">
         <v>938</v>
@@ -2958,7 +2969,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B21" s="8">
         <v>663</v>
@@ -2972,7 +2983,7 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B22" s="8">
         <v>364</v>
@@ -2986,7 +2997,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B23" s="8">
         <v>346</v>
@@ -3000,7 +3011,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B24" s="8">
         <v>371</v>
@@ -3014,7 +3025,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B25" s="8">
         <v>535</v>
@@ -3028,7 +3039,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B26" s="8">
         <v>500</v>
@@ -3042,7 +3053,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B27" s="8">
         <v>756</v>
@@ -3056,7 +3067,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B28" s="8">
         <v>189</v>
@@ -3070,7 +3081,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B29" s="8">
         <v>535</v>
@@ -3084,7 +3095,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B30" s="8">
         <v>253</v>
@@ -3098,7 +3109,7 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B31" s="8">
         <v>299</v>
@@ -3112,7 +3123,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B32" s="8">
         <v>228</v>
@@ -3126,7 +3137,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B33" s="8">
         <v>169</v>
@@ -3140,7 +3151,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B34" s="8">
         <v>76</v>
@@ -3154,7 +3165,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B35" s="8">
         <v>126</v>
@@ -3168,7 +3179,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B36" s="8">
         <v>58</v>
@@ -3182,7 +3193,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B37" s="8">
         <v>94</v>
@@ -3196,7 +3207,7 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B38" s="8">
         <v>61</v>
@@ -3210,7 +3221,7 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B39" s="8">
         <v>34</v>
@@ -3224,7 +3235,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B40" s="8">
         <v>63</v>
@@ -3238,7 +3249,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B41" s="8">
         <v>30</v>
@@ -3252,7 +3263,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B42" s="8">
         <v>54</v>
@@ -3266,7 +3277,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B43" s="8">
         <v>10</v>
@@ -3280,7 +3291,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B44" s="8">
         <v>32</v>
@@ -3315,27 +3326,27 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C2" s="8">
         <v>1446</v>
@@ -3344,15 +3355,15 @@
         <v>322647.47</v>
       </c>
       <c r="E2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C3" s="8">
         <v>43</v>
@@ -3361,15 +3372,15 @@
         <v>-260763.58</v>
       </c>
       <c r="E3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C4" s="8">
         <v>6</v>
@@ -3378,15 +3389,15 @@
         <v>-147614.08</v>
       </c>
       <c r="E4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C5" s="8">
         <v>2122</v>
@@ -3395,15 +3406,15 @@
         <v>112341</v>
       </c>
       <c r="E5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C6" s="8">
         <v>1426</v>
@@ -3412,15 +3423,15 @@
         <v>-82781.26999999999</v>
       </c>
       <c r="E6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C7" s="8">
         <v>102</v>
@@ -3429,15 +3440,15 @@
         <v>-35562.62899999999</v>
       </c>
       <c r="E7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C8" s="8">
         <v>177</v>
@@ -3446,15 +3457,15 @@
         <v>-13484.54</v>
       </c>
       <c r="E8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C9" s="8">
         <v>282</v>
@@ -3463,15 +3474,15 @@
         <v>13386</v>
       </c>
       <c r="E9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C10" s="8">
         <v>16</v>
@@ -3480,15 +3491,15 @@
         <v>-7933.43</v>
       </c>
       <c r="E10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C11" s="8">
         <v>67</v>
@@ -3497,15 +3508,15 @@
         <v>6835.239999999999</v>
       </c>
       <c r="E11" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C12" s="8">
         <v>104</v>
@@ -3514,15 +3525,15 @@
         <v>-6065.8</v>
       </c>
       <c r="E12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C13" s="8">
         <v>3</v>
@@ -3531,15 +3542,15 @@
         <v>731.0500000000001</v>
       </c>
       <c r="E13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C14" s="8">
         <v>29</v>
@@ -3548,15 +3559,15 @@
         <v>610.09</v>
       </c>
       <c r="E14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C15" s="8">
         <v>29</v>
@@ -3565,15 +3576,15 @@
         <v>471.0600000000001</v>
       </c>
       <c r="E15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B16" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C16" s="8">
         <v>25</v>
@@ -3582,15 +3593,15 @@
         <v>295.6300000000001</v>
       </c>
       <c r="E16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C17" s="8">
         <v>15</v>
@@ -3599,15 +3610,15 @@
         <v>292.09</v>
       </c>
       <c r="E17" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B18" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C18" s="8">
         <v>8</v>
@@ -3616,15 +3627,15 @@
         <v>253.59</v>
       </c>
       <c r="E18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C19" s="8">
         <v>23</v>
@@ -3633,15 +3644,15 @@
         <v>251.35</v>
       </c>
       <c r="E19" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B20" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C20" s="8">
         <v>15</v>
@@ -3650,15 +3661,15 @@
         <v>202.5</v>
       </c>
       <c r="E20" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B21" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C21" s="8">
         <v>7</v>
@@ -3667,15 +3678,15 @@
         <v>166.09</v>
       </c>
       <c r="E21" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B22" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C22" s="8">
         <v>16</v>
@@ -3684,15 +3695,15 @@
         <v>126.21</v>
       </c>
       <c r="E22" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B23" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C23" s="8">
         <v>6</v>
@@ -3701,15 +3712,15 @@
         <v>80.31</v>
       </c>
       <c r="E23" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B24" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C24" s="8">
         <v>5</v>
@@ -3718,15 +3729,15 @@
         <v>67.94</v>
       </c>
       <c r="E24" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B25" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C25" s="8">
         <v>3</v>
@@ -3735,15 +3746,15 @@
         <v>59.57</v>
       </c>
       <c r="E25" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B26" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C26" s="8">
         <v>19</v>
@@ -3752,15 +3763,15 @@
         <v>-36.58300000000001</v>
       </c>
       <c r="E26" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B27" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C27" s="8">
         <v>31</v>
@@ -3769,15 +3780,15 @@
         <v>34.82000000000001</v>
       </c>
       <c r="E27" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B28" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C28" s="8">
         <v>14</v>
@@ -3786,15 +3797,15 @@
         <v>32.59</v>
       </c>
       <c r="E28" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B29" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C29" s="8">
         <v>3</v>
@@ -3803,15 +3814,15 @@
         <v>25.44</v>
       </c>
       <c r="E29" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B30" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C30" s="8">
         <v>4</v>
@@ -3820,15 +3831,15 @@
         <v>20.68</v>
       </c>
       <c r="E30" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B31" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C31" s="8">
         <v>4</v>
@@ -3837,15 +3848,15 @@
         <v>17.3</v>
       </c>
       <c r="E31" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B32" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C32" s="8">
         <v>3</v>
@@ -3854,15 +3865,15 @@
         <v>17.12</v>
       </c>
       <c r="E32" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B33" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C33" s="8">
         <v>3</v>
@@ -3871,15 +3882,15 @@
         <v>14.75</v>
       </c>
       <c r="E33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B34" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C34" s="8">
         <v>2</v>
@@ -3888,15 +3899,15 @@
         <v>12.72</v>
       </c>
       <c r="E34" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B35" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C35" s="8">
         <v>1</v>
@@ -3905,15 +3916,15 @@
         <v>12.72</v>
       </c>
       <c r="E35" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B36" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C36" s="8">
         <v>1</v>
@@ -3922,15 +3933,15 @@
         <v>5.06</v>
       </c>
       <c r="E36" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B37" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C37" s="8">
         <v>1</v>
@@ -3939,15 +3950,15 @@
         <v>2.57</v>
       </c>
       <c r="E37" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B38" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C38" s="8">
         <v>2</v>
@@ -3956,15 +3967,15 @@
         <v>2.51</v>
       </c>
       <c r="E38" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B39" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C39" s="8">
         <v>2</v>
@@ -3973,15 +3984,15 @@
         <v>1</v>
       </c>
       <c r="E39" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B40" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C40" s="8">
         <v>1</v>
@@ -3992,10 +4003,10 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B41" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C41" s="8">
         <v>1</v>
@@ -4006,10 +4017,10 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B42" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C42" s="8">
         <v>1</v>
@@ -4020,10 +4031,10 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B43" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C43" s="8">
         <v>1</v>
@@ -4034,10 +4045,10 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B44" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C44" s="8">
         <v>1</v>
@@ -4048,10 +4059,10 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B45" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C45" s="8">
         <v>1</v>
@@ -4062,10 +4073,10 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B46" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C46" s="8">
         <v>1</v>
@@ -4076,10 +4087,10 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B47" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C47" s="8">
         <v>1</v>
@@ -4090,10 +4101,10 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B48" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C48" s="8">
         <v>1</v>
@@ -4104,10 +4115,10 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B49" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C49" s="8">
         <v>1</v>
@@ -4118,10 +4129,10 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B50" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C50" s="8">
         <v>1</v>
@@ -4132,10 +4143,10 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B51" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C51" s="8">
         <v>1</v>
@@ -4146,10 +4157,10 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B52" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C52" s="8">
         <v>1</v>
@@ -4160,10 +4171,10 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B53" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C53" s="8">
         <v>1</v>
@@ -4172,15 +4183,15 @@
         <v>0</v>
       </c>
       <c r="E53" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B54" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C54" s="8">
         <v>1</v>
@@ -4191,10 +4202,10 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B55" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C55" s="8">
         <v>1</v>
@@ -4205,10 +4216,10 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B56" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C56" s="8">
         <v>1</v>
@@ -4219,10 +4230,10 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B57" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C57" s="8">
         <v>1</v>
@@ -4233,10 +4244,10 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B58" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C58" s="8">
         <v>1</v>
@@ -4247,10 +4258,10 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B59" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C59" s="8">
         <v>1</v>
@@ -4259,15 +4270,15 @@
         <v>0</v>
       </c>
       <c r="E59" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B60" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C60" s="8">
         <v>2</v>
@@ -4278,10 +4289,10 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B61" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C61" s="8">
         <v>4</v>
@@ -4290,15 +4301,15 @@
         <v>0</v>
       </c>
       <c r="E61" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B62" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C62" s="8">
         <v>2</v>

</xml_diff>